<commit_message>
Add explicit Save to Google Sheet option, buttons, and live sync handling
</commit_message>
<xml_diff>
--- a/server/data/monthly-website-reports.xlsx
+++ b/server/data/monthly-website-reports.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="100">
   <si>
     <t>WORDPRESS MAINTENANCE &amp; SECURITY COMPLIANCE MATRIX</t>
   </si>
@@ -56,19 +56,25 @@
     <t>Overall %</t>
   </si>
   <si>
+    <t>https://behavirolahealthmarketing.com</t>
+  </si>
+  <si>
+    <t>DONE</t>
+  </si>
+  <si>
+    <t>DONE (8.4)</t>
+  </si>
+  <si>
+    <t>100%</t>
+  </si>
+  <si>
     <t>https://webdesignshop.com</t>
   </si>
   <si>
-    <t>DONE</t>
-  </si>
-  <si>
     <t>DONE (PHP 8.2)</t>
   </si>
   <si>
-    <t>DONE (v6.7.1)</t>
-  </si>
-  <si>
-    <t>100%</t>
+    <t>DONE (6.7.1)</t>
   </si>
   <si>
     <t>https://with-selected-versions-test.com</t>
@@ -92,12 +98,6 @@
     <t>https://wphide-test-client.com</t>
   </si>
   <si>
-    <t>UNDONE (PHP 8.2)</t>
-  </si>
-  <si>
-    <t>UNDONE (v6.7.1)</t>
-  </si>
-  <si>
     <t>10%</t>
   </si>
   <si>
@@ -155,6 +155,27 @@
     <t>Created Timestamp</t>
   </si>
   <si>
+    <t>d764c3ac-142f-479e-8a84-7e709f7279e7</t>
+  </si>
+  <si>
+    <t>Behavirolahealthmarketing</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>This report summarizes the WordPress maintenance, upgrade, security configuration, email delivery, and quality assurance tasks recorded for behavirolahealthmarketing.com as of 2026-10-29. All scheduled maintenance, upgrade, and verification items have been successfully executed.</t>
+  </si>
+  <si>
+    <t>All 10 recorded maintenance tasks for this website are marked as completed, achieving a 100% completion rate. All core, plugin, theme, and security checks have been documented and fulfilled.</t>
+  </si>
+  <si>
+    <t>None recorded</t>
+  </si>
+  <si>
+    <t>2026-10-29T16:51:03.385Z</t>
+  </si>
+  <si>
     <t>73943f92-23cf-44e9-a96a-a8fe781eeb65</t>
   </si>
   <si>
@@ -165,12 +186,6 @@
   </si>
   <si>
     <t>This report summarizes the WordPress maintenance, upgrade, security configuration, email delivery, and quality assurance tasks recorded for webdesignshop.com as of 2026-10-28. All scheduled maintenance, upgrade, and verification items have been successfully executed.</t>
-  </si>
-  <si>
-    <t>All 10 recorded maintenance tasks for this website are marked as completed, achieving a 100% completion rate. All core, plugin, theme, and security checks have been documented and fulfilled.</t>
-  </si>
-  <si>
-    <t>None recorded</t>
   </si>
   <si>
     <t>2026-10-28T16:22:01.700Z</t>
@@ -751,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -850,13 +865,13 @@
         <v>15</v>
       </c>
       <c r="K3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M3" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -864,40 +879,40 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="G4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="5" t="s">
+      <c r="L4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -905,37 +920,37 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="G5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="L5" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M5" s="6" t="s">
         <v>24</v>
@@ -949,37 +964,37 @@
         <v>25</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -987,40 +1002,40 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>15</v>
+        <v>27</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>30</v>
+        <v>22</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1028,34 +1043,34 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>30</v>
@@ -1069,40 +1084,40 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>15</v>
+      <c r="D9" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>30</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1110,7 +1125,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>15</v>
@@ -1118,11 +1133,11 @@
       <c r="D10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>15</v>
+      <c r="E10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>15</v>
@@ -1130,20 +1145,61 @@
       <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>15</v>
+      <c r="I10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="5" t="s">
-        <v>18</v>
+      <c r="M10" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1157,7 +1213,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1234,7 +1290,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>50</v>
@@ -1254,7 +1310,7 @@
         <v>54</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>55</v>
@@ -1263,22 +1319,22 @@
         <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F3" s="3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G3" s="3">
         <v>10</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>52</v>
@@ -1292,7 +1348,7 @@
         <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>60</v>
@@ -1301,10 +1357,10 @@
         <v>30</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F4" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4" s="3">
         <v>10</v>
@@ -1339,16 +1395,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3">
         <v>10</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>66</v>
@@ -1368,7 +1424,7 @@
         <v>69</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>70</v>
@@ -1377,16 +1433,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F6" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>71</v>
@@ -1406,16 +1462,16 @@
         <v>74</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>75</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F7" s="3">
         <v>2</v>
@@ -1427,92 +1483,130 @@
         <v>31</v>
       </c>
       <c r="I7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>72</v>
-      </c>
       <c r="K7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="3">
+        <v>2</v>
+      </c>
+      <c r="G8" s="3">
+        <v>9</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="3">
-        <v>9</v>
-      </c>
-      <c r="G8" s="3">
-        <v>12</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>89</v>
-      </c>
       <c r="E9" s="3" t="s">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="F9" s="3">
         <v>9</v>
       </c>
       <c r="G9" s="3">
+        <v>12</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F10" s="3">
         <v>9</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>94</v>
+      <c r="G10" s="3">
+        <v>9</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>